<commit_message>
Make General Tasks a continuation with a light separator
</commit_message>
<xml_diff>
--- a/Central_50_Task_Sheet.xlsx
+++ b/Central_50_Task_Sheet.xlsx
@@ -51,8 +51,9 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="13"/>
+      <i val="1"/>
+      <color rgb="00305496"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="9">
@@ -94,11 +95,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007F7F7F"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -120,11 +121,25 @@
         <color rgb="00999999"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="medium">
+        <color rgb="00305496"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -177,9 +192,10 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -551,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -885,130 +901,102 @@
       <c r="E24" s="17" t="n"/>
       <c r="F24" s="17" t="n"/>
     </row>
-    <row r="25" ht="18" customHeight="1"/>
-    <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>GENERAL TASKS</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Brand Name</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Date of Raise</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Assign</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>Date Due for Completion</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>General Tasks</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="n"/>
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+      <c r="F25" s="19" t="n"/>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="20" t="inlineStr"/>
+      <c r="B26" s="20" t="inlineStr"/>
+      <c r="C26" s="21" t="inlineStr"/>
+      <c r="D26" s="21" t="inlineStr"/>
+      <c r="E26" s="21" t="inlineStr"/>
+      <c r="F26" s="21" t="inlineStr"/>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="20" t="inlineStr"/>
+      <c r="B27" s="20" t="inlineStr"/>
+      <c r="C27" s="21" t="inlineStr"/>
+      <c r="D27" s="21" t="inlineStr"/>
+      <c r="E27" s="21" t="inlineStr"/>
+      <c r="F27" s="21" t="inlineStr"/>
     </row>
     <row r="28" ht="42" customHeight="1">
-      <c r="A28" s="19" t="inlineStr"/>
-      <c r="B28" s="19" t="inlineStr"/>
-      <c r="C28" s="20" t="inlineStr"/>
-      <c r="D28" s="20" t="inlineStr"/>
-      <c r="E28" s="20" t="inlineStr"/>
-      <c r="F28" s="20" t="inlineStr"/>
+      <c r="A28" s="20" t="inlineStr"/>
+      <c r="B28" s="20" t="inlineStr"/>
+      <c r="C28" s="21" t="inlineStr"/>
+      <c r="D28" s="21" t="inlineStr"/>
+      <c r="E28" s="21" t="inlineStr"/>
+      <c r="F28" s="21" t="inlineStr"/>
     </row>
     <row r="29" ht="42" customHeight="1">
-      <c r="A29" s="19" t="inlineStr"/>
-      <c r="B29" s="19" t="inlineStr"/>
-      <c r="C29" s="20" t="inlineStr"/>
-      <c r="D29" s="20" t="inlineStr"/>
-      <c r="E29" s="20" t="inlineStr"/>
-      <c r="F29" s="20" t="inlineStr"/>
+      <c r="A29" s="20" t="inlineStr"/>
+      <c r="B29" s="20" t="inlineStr"/>
+      <c r="C29" s="21" t="inlineStr"/>
+      <c r="D29" s="21" t="inlineStr"/>
+      <c r="E29" s="21" t="inlineStr"/>
+      <c r="F29" s="21" t="inlineStr"/>
     </row>
     <row r="30" ht="42" customHeight="1">
-      <c r="A30" s="19" t="inlineStr"/>
-      <c r="B30" s="19" t="inlineStr"/>
-      <c r="C30" s="20" t="inlineStr"/>
-      <c r="D30" s="20" t="inlineStr"/>
-      <c r="E30" s="20" t="inlineStr"/>
-      <c r="F30" s="20" t="inlineStr"/>
+      <c r="A30" s="20" t="inlineStr"/>
+      <c r="B30" s="20" t="inlineStr"/>
+      <c r="C30" s="21" t="inlineStr"/>
+      <c r="D30" s="21" t="inlineStr"/>
+      <c r="E30" s="21" t="inlineStr"/>
+      <c r="F30" s="21" t="inlineStr"/>
     </row>
     <row r="31" ht="42" customHeight="1">
-      <c r="A31" s="19" t="inlineStr"/>
-      <c r="B31" s="19" t="inlineStr"/>
-      <c r="C31" s="20" t="inlineStr"/>
-      <c r="D31" s="20" t="inlineStr"/>
-      <c r="E31" s="20" t="inlineStr"/>
-      <c r="F31" s="20" t="inlineStr"/>
+      <c r="A31" s="20" t="inlineStr"/>
+      <c r="B31" s="20" t="inlineStr"/>
+      <c r="C31" s="21" t="inlineStr"/>
+      <c r="D31" s="21" t="inlineStr"/>
+      <c r="E31" s="21" t="inlineStr"/>
+      <c r="F31" s="21" t="inlineStr"/>
     </row>
     <row r="32" ht="42" customHeight="1">
-      <c r="A32" s="19" t="inlineStr"/>
-      <c r="B32" s="19" t="inlineStr"/>
-      <c r="C32" s="20" t="inlineStr"/>
-      <c r="D32" s="20" t="inlineStr"/>
-      <c r="E32" s="20" t="inlineStr"/>
-      <c r="F32" s="20" t="inlineStr"/>
+      <c r="A32" s="20" t="inlineStr"/>
+      <c r="B32" s="20" t="inlineStr"/>
+      <c r="C32" s="21" t="inlineStr"/>
+      <c r="D32" s="21" t="inlineStr"/>
+      <c r="E32" s="21" t="inlineStr"/>
+      <c r="F32" s="21" t="inlineStr"/>
     </row>
     <row r="33" ht="42" customHeight="1">
-      <c r="A33" s="19" t="inlineStr"/>
-      <c r="B33" s="19" t="inlineStr"/>
-      <c r="C33" s="20" t="inlineStr"/>
-      <c r="D33" s="20" t="inlineStr"/>
-      <c r="E33" s="20" t="inlineStr"/>
-      <c r="F33" s="20" t="inlineStr"/>
+      <c r="A33" s="20" t="inlineStr"/>
+      <c r="B33" s="20" t="inlineStr"/>
+      <c r="C33" s="21" t="inlineStr"/>
+      <c r="D33" s="21" t="inlineStr"/>
+      <c r="E33" s="21" t="inlineStr"/>
+      <c r="F33" s="21" t="inlineStr"/>
     </row>
     <row r="34" ht="42" customHeight="1">
-      <c r="A34" s="19" t="inlineStr"/>
-      <c r="B34" s="19" t="inlineStr"/>
-      <c r="C34" s="20" t="inlineStr"/>
-      <c r="D34" s="20" t="inlineStr"/>
-      <c r="E34" s="20" t="inlineStr"/>
-      <c r="F34" s="20" t="inlineStr"/>
+      <c r="A34" s="20" t="inlineStr"/>
+      <c r="B34" s="20" t="inlineStr"/>
+      <c r="C34" s="21" t="inlineStr"/>
+      <c r="D34" s="21" t="inlineStr"/>
+      <c r="E34" s="21" t="inlineStr"/>
+      <c r="F34" s="21" t="inlineStr"/>
     </row>
     <row r="35" ht="42" customHeight="1">
-      <c r="A35" s="19" t="inlineStr"/>
-      <c r="B35" s="19" t="inlineStr"/>
-      <c r="C35" s="20" t="inlineStr"/>
-      <c r="D35" s="20" t="inlineStr"/>
-      <c r="E35" s="20" t="inlineStr"/>
-      <c r="F35" s="20" t="inlineStr"/>
-    </row>
-    <row r="36" ht="42" customHeight="1">
-      <c r="A36" s="19" t="inlineStr"/>
-      <c r="B36" s="19" t="inlineStr"/>
-      <c r="C36" s="20" t="inlineStr"/>
-      <c r="D36" s="20" t="inlineStr"/>
-      <c r="E36" s="20" t="inlineStr"/>
-      <c r="F36" s="20" t="inlineStr"/>
-    </row>
-    <row r="37" ht="42" customHeight="1">
-      <c r="A37" s="19" t="inlineStr"/>
-      <c r="B37" s="19" t="inlineStr"/>
-      <c r="C37" s="20" t="inlineStr"/>
-      <c r="D37" s="20" t="inlineStr"/>
-      <c r="E37" s="20" t="inlineStr"/>
-      <c r="F37" s="20" t="inlineStr"/>
+      <c r="A35" s="20" t="inlineStr"/>
+      <c r="B35" s="20" t="inlineStr"/>
+      <c r="C35" s="21" t="inlineStr"/>
+      <c r="D35" s="21" t="inlineStr"/>
+      <c r="E35" s="21" t="inlineStr"/>
+      <c r="F35" s="21" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>